<commit_message>
Update data plan workbook after enabling full network access
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019genJUXM7TYZhfbpNvVXCS
</commit_message>
<xml_diff>
--- a/FantaBall-Complete/docs/Data-Sources-and-Calibration-Plan.xlsx
+++ b/FantaBall-Complete/docs/Data-Sources-and-Calibration-Plan.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="506">
   <si>
     <t xml:space="preserve">FantaBall — data sources and calibration plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Prepared 23-Oct-2026. Connectivity tested from the Claude Code cloud environment that day.</t>
+    <t xml:space="preserve">Prepared 23-Oct-2026. Connectivity re-tested the same day after network access was set to allow all.</t>
   </si>
   <si>
     <t xml:space="preserve">Data items</t>
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Key / login needed</t>
   </si>
   <si>
-    <t xml:space="preserve">Reachable from this cloud env (tested 23-Oct-2026)</t>
+    <t xml:space="preserve">Reachable from this cloud env (re-tested 23-Oct-2026, full access)</t>
   </si>
   <si>
     <t xml:space="preserve">Solvable with no input from you?</t>
@@ -174,7 +174,7 @@
     <t xml:space="preserve">Season start; check after promotions</t>
   </si>
   <si>
-    <t xml:space="preserve">Community-maintained. Cross-check names against a second source once one is reachable.</t>
+    <t xml:space="preserve">Cross-checked against the Fantacalcio.it list and football-data.co.uk.</t>
   </si>
   <si>
     <t xml:space="preserve">T2</t>
@@ -198,7 +198,7 @@
     <t xml:space="preserve">Weekly (postponements)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lags by a few days; postponed matches need a second source to confirm.</t>
+    <t xml:space="preserve">football-data.co.uk fixtures.csv confirms dates for the coming week.</t>
   </si>
   <si>
     <t xml:space="preserve">T3</t>
@@ -213,7 +213,7 @@
     <t xml:space="preserve">Not used</t>
   </si>
   <si>
-    <t xml:space="preserve">GitHub openfootball (raw.githubusercontent.com) it.1.json / italy/*.txt</t>
+    <t xml:space="preserve">football-data.co.uk I1.csv (results, shots, cards, odds) + openfootball</t>
   </si>
   <si>
     <t xml:space="preserve">football-data.co.uk I1.csv</t>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">Weekly</t>
   </si>
   <si>
-    <t xml:space="preserve">About 50 of the 2026/27 results were present on 23-Oct (lags 1–3 matchdays).</t>
+    <t xml:space="preserve">Current and past seasons available.</t>
   </si>
   <si>
     <t xml:space="preserve">T4</t>
@@ -240,7 +240,7 @@
     <t xml:space="preserve">High</t>
   </si>
   <si>
-    <t xml:space="preserve">The Odds API</t>
+    <t xml:space="preserve">football-data.co.uk (closing odds for played matches; fixtures.csv has odds for the coming matchday)</t>
   </si>
   <si>
     <t xml:space="preserve">football-data.co.uk (closing odds in I1.csv)</t>
@@ -252,16 +252,10 @@
     <t xml:space="preserve">The Odds API: free key</t>
   </si>
   <si>
-    <t xml:space="preserve">No (403)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fit team strengths from results only (T3).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow domain(s) + optional API key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Odds are the most accurate public team-strength signal.</t>
+    <t xml:space="preserve">— (The Odds API key optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upcoming odds cover about one matchday ahead; later fixtures use the results/xG model.</t>
   </si>
   <si>
     <t xml:space="preserve">T5</t>
@@ -276,402 +270,351 @@
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
+    <t xml:space="preserve">Understat getLeagueData (teams)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrape embedded JSON / HTML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBref is behind a Cloudflare bot check even in a headless browser; Understat replaces it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Club Elo ratings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior for team strength / promoted clubs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">api.clubelo.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSV API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No (connection drops)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not needed: odds + xG cover team strength.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— (optional, dropped)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional; can be removed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formation / coach per team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MODEL.formation (currently one 4-3-3 for all)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed 4-3-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it probabili formazioni (module) + Understat match logs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it probabili formazioni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep 4-3-3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Player</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Player list per club with official Fantacalcio role (P/D/C/A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[] id, name, team, role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthetic 18 per club</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it quotazioni (603 players, Classic and Mantra roles, QI/QA/FVM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio-online, FBref squad pages (no Fantacalcio roles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrape / Excel download</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel export may need a free login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly (transfers, role changes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parsed from page HTML; no login needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfers in/out, squad changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it listone diff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfermarkt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diff of weekly listone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detected by diffing P1 week to week.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly; daily in transfer windows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfermarkt (headless browser) as a second check.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Match votes (voto) and fantavoto per player per match, current + 2–3 past seasons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].base; MODEL.vote.* (win, loss, goalDiff, teamSd, indivSd, goal, assist, red, gk/def conceded &amp; clean); subRatedMin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthetic 5.9–6.4; coefficients guessed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it voti per giornata (current and past seasons; Fantacalcio, Statistico and Italia votes; bonus/malus detail)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio-online match pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrape per matchday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly (after each matchday)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Includes goals, conceded, own goals, penalties scored/missed/saved, cards per player.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goals per player incl. penalties and own goals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].goalW; MODEL.ownGoal; penalty share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthetic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it voti (bonus detail) + Understat (goals, npg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBref, API-Football, fantacalcio.it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parse text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assists per player</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].assistW; MODEL.assisted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understat (assists, xA) + Fantacalcio.it voti (Fantacalcio assists)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-Football, Understat, fantacalcio.it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrape / API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-Football: free key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio assists are what the league scores; Understat gives per-90 rates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minutes, starts and substitute appearances per match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].start; goalW/assistW per 90; MODEL.subs, subMinutes, subRatedMin; formation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understat getPlayerData (per-match minutes; start vs "Sub")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-Football fixtures/players, fantacalcio.it tabellini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About 600 player requests per full refresh; throttled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xG / xA / shots per player</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shrinkage prior for goalW/assistW (less noise than goals)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Understat</t>
   </si>
   <si>
-    <t xml:space="preserve">FBref</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scrape embedded JSON / HTML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use goals only (T3).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Personal use only; check site terms.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Club Elo ratings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior for team strength / promoted clubs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low</t>
-  </si>
-  <si>
-    <t xml:space="preserve">api.clubelo.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSV API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Promoted clubs get a league-average-minus prior.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formation / coach per team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MODEL.formation (currently one 4-3-3 for all)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed 4-3-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derived from lineups (P6/P13)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio.it probabili formazioni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derived</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep 4-3-3.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow fantacalcio.it or fbref</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coach changes trigger a refit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Player</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Player list per club with official Fantacalcio role (P/D/C/A)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[] id, name, team, role</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Synthetic 18 per club</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio.it quotazioni/listone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio-online, FBref squad pages (no Fantacalcio roles)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scrape / Excel download</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excel export may need a free login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None credible: roles are set by the game provider.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly (transfers, role changes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow fantacalcio.it (or provide login secret if export needs it)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Without this the model cannot simulate real players.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transfers in/out, squad changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio.it listone diff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transfermarkt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diff of weekly listone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Detected by diffing P1 week to week.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly; daily in transfer windows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Match votes (voto) and fantavoto per player per match, current + 2–3 past seasons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].base; MODEL.vote.* (win, loss, goalDiff, teamSd, indivSd, goal, assist, red, gk/def conceded &amp; clean); subRatedMin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Synthetic 5.9–6.4; coefficients guessed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio.it voti per giornata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio-online match pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scrape per matchday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No (DNS blocked / 403)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Role-average base 6.0; coefficients stay at guesses.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly (after each matchday)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow fantacalcio.it (and/or fantacalcio-online.com)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vote provider must match your league (Fantacalcio.it / Statistico / Italia).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goals per player incl. penalties and own goals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].goalW; MODEL.ownGoal; penalty share</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Synthetic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GitHub openfootball (raw.githubusercontent.com) italy/*.txt (scorers with (p) and (og) markers)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FBref, API-Football, fantacalcio.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parse text</t>
+    <t xml:space="preserve">Scrape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penalty takers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penalty share inside goalW (planned penalty model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not modelled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it rigoristi + penalty detail in voti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it rigoristi page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow and red cards per player</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].yellow; MODEL.red; suspensions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Synthetic by role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understat + Fantacalcio.it voti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API-Football, fantacalcio.it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current injuries and expected return date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].injuredFor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Random 6% injured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it indisponibili + Transfermarkt injured players (headless browser)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfermarkt injuries, club news</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly + on news</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text return dates converted to matches missed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Injury history (frequency and length)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].injuryRisk, injuryGames</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfermarkt player injury history (headless browser)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FBref (missed matches)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (browser only)</t>
   </si>
   <si>
     <t xml:space="preserve">Partial</t>
   </si>
   <si>
-    <t xml:space="preserve">Goal counts available, but no minutes to turn them into per-90 rates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">— (full rates need P6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name matching to P1 is needed once rosters exist.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assists per player</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].assistW; MODEL.assisted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-Football, Understat, fantacalcio.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scrape / API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-Football: free key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Role-average assist share.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow domain or API key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio assists differ slightly from Opta assists.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minutes, starts and substitute appearances per match</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].start; goalW/assistW per 90; MODEL.subs, subMinutes, subRatedMin; formation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FBref match logs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-Football fixtures/players, fantacalcio.it tabellini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None good: titolarità is a key driver.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow fbref.com or API key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xG / xA / shots per player</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shrinkage prior for goalW/assistW (less noise than goals)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scrape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use goals/assists only, with stronger shrinkage to role means.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Penalty takers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Penalty share inside goalW (planned penalty model)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not modelled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derived from P4 (p) markers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio.it rigoristi page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Infer from past penalty scorers; misses not visible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow fantacalcio.it for missed penalties</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow and red cards per player</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].yellow; MODEL.red; suspensions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Synthetic by role</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API-Football, fantacalcio.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Role-average card rates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current injuries and expected return date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].injuredFor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Random 6% injured</t>
+    <t xml:space="preserve">Age/role priors for players without history.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bot protection: slow, throttled scraping of ~600 pages; refresh monthly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current suspensions and yellow-card count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">players[].yellows; banned at start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zero for all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it squalificati e diffidati + card counts</t>
   </si>
   <si>
     <t xml:space="preserve">Fantacalcio.it indisponibili</t>
   </si>
   <si>
-    <t xml:space="preserve">Transfermarkt injuries, club news</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No (DNS blocked)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Everyone treated as fit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly + on news</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow fantacalcio.it or transfermarkt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Text return dates need converting to matches missed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Injury history (frequency and length)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].injuryRisk, injuryGames</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transfermarkt injury history</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FBref (missed matches)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age/role priors from published injury studies.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow transfermarkt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current suspensions and yellow-card count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">players[].yellows; banned at start</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zero for all</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derived from P9 + official disciplinary decisions</t>
-  </si>
-  <si>
     <t xml:space="preserve">Derived / scrape</t>
   </si>
   <si>
-    <t xml:space="preserve">Count from P9 once available.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same as P9/P10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The suspension thresholds are a regulation; confirm once (see Model_Parameters).</t>
-  </si>
-  <si>
     <t xml:space="preserve">P13</t>
   </si>
   <si>
@@ -684,15 +627,9 @@
     <t xml:space="preserve">Sky Sport, Gazzetta probabili</t>
   </si>
   <si>
-    <t xml:space="preserve">Use season-long start weights (P6).</t>
-  </si>
-  <si>
     <t xml:space="preserve">Before each matchday</t>
   </si>
   <si>
-    <t xml:space="preserve">Allow fantacalcio.it</t>
-  </si>
-  <si>
     <t xml:space="preserve">L1</t>
   </si>
   <si>
@@ -795,7 +732,7 @@
     <t xml:space="preserve">P6, T7</t>
   </si>
   <si>
-    <t xml:space="preserve">Guess</t>
+    <t xml:space="preserve">Guess — data now reachable</t>
   </si>
   <si>
     <t xml:space="preserve">baseGoals</t>
@@ -852,6 +789,9 @@
     <t xml:space="preserve">T3, T4, T5, T6</t>
   </si>
   <si>
+    <t xml:space="preserve">Synthetic — data now reachable</t>
+  </si>
+  <si>
     <t xml:space="preserve">teamSd</t>
   </si>
   <si>
@@ -1266,16 +1206,16 @@
     <t xml:space="preserve">Host</t>
   </si>
   <si>
-    <t xml:space="preserve">What it would provide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">curl from container</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude WebFetch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Result</t>
+    <t xml:space="preserve">What it provides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plain request from container</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Headless browser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usable</t>
   </si>
   <si>
     <t xml:space="preserve">raw.githubusercontent.com (openfootball)</t>
@@ -1290,13 +1230,10 @@
     <t xml:space="preserve">www.fantacalcio.it</t>
   </si>
   <si>
-    <t xml:space="preserve">Roles, votes, injuries, probable lineups</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked (proxy 403)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNS not resolved</t>
+    <t xml:space="preserve">Roles (603 players), votes per match, injuries, suspensions, probable lineups</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 OK, data in page HTML</t>
   </si>
   <si>
     <t xml:space="preserve">www.fantacalcio-online.com</t>
@@ -1305,16 +1242,34 @@
     <t xml:space="preserve">Votes per match (backup)</t>
   </si>
   <si>
-    <t xml:space="preserve">Not tested</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Untested (same policy blocks it)</t>
-  </si>
-  <si>
     <t xml:space="preserve">www.football-data.co.uk</t>
   </si>
   <si>
-    <t xml:space="preserve">Results, cards, closing odds</t>
+    <t xml:space="preserve">Results, cards, shots, closing odds; odds for the coming matchday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 OK (after redirect)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">understat.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-player season and per-match minutes, starts/sub, goals, xG, assists, xA, cards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 OK (JSON endpoints)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">www.transfermarkt.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Injuries, injury history, transfers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">405 to plain requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 OK in headless Chromium</t>
   </si>
   <si>
     <t xml:space="preserve">fbref.com</t>
@@ -1323,46 +1278,34 @@
     <t xml:space="preserve">Minutes, assists, cards, xG</t>
   </si>
   <si>
-    <t xml:space="preserve">understat.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xG / xA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">www.transfermarkt.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Injuries, transfers</t>
+    <t xml:space="preserve">403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloudflare challenge in headless Chromium</t>
   </si>
   <si>
     <t xml:space="preserve">Elo ratings</t>
   </si>
   <si>
+    <t xml:space="preserve">Connection dropped</t>
+  </si>
+  <si>
     <t xml:space="preserve">v3.football.api-sports.io</t>
   </si>
   <si>
     <t xml:space="preserve">API-Football (structured stats)</t>
   </si>
   <si>
+    <t xml:space="preserve">Reachable (403 = no key)</t>
+  </si>
+  <si>
     <t xml:space="preserve">api.the-odds-api.com</t>
   </si>
   <si>
     <t xml:space="preserve">Betting odds</t>
   </si>
   <si>
-    <t xml:space="preserve">api.sofascore.com / fotmob.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lineups, ratings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Web search</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finding pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Works (titles and snippets only)</t>
+    <t xml:space="preserve">Reachable (401 = no key)</t>
   </si>
   <si>
     <t xml:space="preserve">Step</t>
@@ -1431,7 +1374,7 @@
     <t xml:space="preserve">Engine runs on real clubs and calendar</t>
   </si>
   <si>
-    <t xml:space="preserve">B — after domains allowed</t>
+    <t xml:space="preserve">B — now unblocked</t>
   </si>
   <si>
     <t xml:space="preserve">Rosters and roles</t>
@@ -1458,15 +1401,12 @@
     <t xml:space="preserve">data/raw/votes/*.csv</t>
   </si>
   <si>
-    <t xml:space="preserve">Scrape FBref match logs + Understat (or call API-Football with a key)</t>
+    <t xml:space="preserve">Understat season + per-match player data (FBref blocked by Cloudflare, not needed)</t>
   </si>
   <si>
     <t xml:space="preserve">P5, P6, P7, P9</t>
   </si>
   <si>
-    <t xml:space="preserve">Allow fbref.com and understat.com, or add API-Football key</t>
-  </si>
-  <si>
     <t xml:space="preserve">data/raw/player_matches.csv</t>
   </si>
   <si>
@@ -1485,10 +1425,10 @@
     <t xml:space="preserve">Odds</t>
   </si>
   <si>
-    <t xml:space="preserve">Fetch match odds; blend with results-based team strengths</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allow football-data.co.uk or add The Odds API key</t>
+    <t xml:space="preserve">football-data.co.uk odds (played + coming matchday); blend with results/xG team strengths</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None (Odds API key optional)</t>
   </si>
   <si>
     <t xml:space="preserve">data/raw/odds_&lt;date&gt;.csv</t>
@@ -1551,46 +1491,49 @@
     <t xml:space="preserve">How (one-time)</t>
   </si>
   <si>
-    <t xml:space="preserve">Allow these domains in the cloud environment network settings: www.fantacalcio.it, fbref.com, understat.com, www.football-data.co.uk, www.transfermarkt.com (or switch the environment to full network access)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every player-level source is blocked here; only GitHub is reachable. Without this, phases B–D cannot run and players stay synthetic.</t>
+    <t xml:space="preserve">Network access set to allow all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unblocked every source the plan needs (FBref replaced by Understat).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Done on 23-Oct-2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional API keys saved as environment secrets: API_FOOTBALL_KEY (api-sports.io), ODDS_API_KEY (the-odds-api.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not needed now; would add odds for fixtures beyond the coming matchday and a structured backup if scraping breaks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create free accounts, add the keys as environment variables.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm the league rules not yet captured: vote provider (Fantacalcio / Statistico / Italia), defence modifier formula, penalty scored/missed/saved, own goal, no-vote rule, Classic vs Mantra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The simulation must score exactly as your league does. This is the only item that blocks a fully calibrated model.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required (once)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer once; stored in a config file in the repo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm personal (non-commercial) use of scraped data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fantacalcio.it, Understat and Transfermarkt terms restrict automated and commercial reuse; a commercial app needs a licensed feed.</t>
   </si>
   <si>
     <t xml:space="preserve">Required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Environment settings → Network access → add Allowed domains (keep "Allow package managers" ticked).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional API keys saved as environment secrets: API_FOOTBALL_KEY (api-sports.io free tier), ODDS_API_KEY (the-odds-api.com free tier) and their domains allowed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structured APIs are more stable than scraping; odds improve team strengths.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create free accounts, add the keys as environment variables.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm the league rules not yet captured: vote provider, defence modifier formula, penalty scored/missed/saved, own goal, no-vote rule, Classic vs Mantra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The simulation must score exactly as your league does.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Required (once)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Answer once; stored in a config file in the repo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm personal (non-commercial) use of scraped data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fantacalcio.it, FBref and Transfermarkt terms restrict automated and commercial reuse; a commercial app needs a licensed feed.</t>
   </si>
   <si>
     <t xml:space="preserve">A yes/no answer.</t>
@@ -1898,14 +1841,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Connectivity" displayName="Connectivity" ref="A1:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:E13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Connectivity" displayName="Connectivity" ref="A1:E11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E11"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Host"/>
-    <tableColumn id="2" name="What it would provide"/>
-    <tableColumn id="3" name="curl from container"/>
-    <tableColumn id="4" name="Claude WebFetch"/>
-    <tableColumn id="5" name="Result"/>
+    <tableColumn id="2" name="What it provides"/>
+    <tableColumn id="3" name="Plain request from container"/>
+    <tableColumn id="4" name="Headless browser"/>
+    <tableColumn id="5" name="Usable"/>
   </tableColumns>
 </table>
 </file>
@@ -1924,7 +1867,7 @@
     <tableColumn id="8" name="Backup source(s)"/>
     <tableColumn id="9" name="Access method"/>
     <tableColumn id="10" name="Key / login needed"/>
-    <tableColumn id="11" name="Reachable from this cloud env (tested 23-Oct-2026)"/>
+    <tableColumn id="11" name="Reachable from this cloud env (re-tested 23-Oct-2026, full access)"/>
     <tableColumn id="12" name="Solvable with no input from you?"/>
     <tableColumn id="13" name="Fallback / imputation if unavailable"/>
     <tableColumn id="14" name="Refresh cadence"/>
@@ -2190,7 +2133,7 @@
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">COUNTIF(Data_Sources!L:L,"Yes")</f>
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2199,7 +2142,7 @@
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">COUNTIF(Data_Sources!L:L,"Partial")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2208,7 +2151,7 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">COUNTIF(Data_Sources!L:L,"No")</f>
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2226,7 +2169,7 @@
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">COUNTIFS(Data_Sources!F:F,"Critical",Data_Sources!L:L,"No")</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2247,7 +2190,7 @@
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">COUNTIF(Model_Parameters!H:H,"Yes")</f>
-        <v>6</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2256,7 +2199,7 @@
       </c>
       <c r="B13" s="4" t="n">
         <f aca="false">COUNTIF(Model_Parameters!H:H,"Partial")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2265,7 +2208,7 @@
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">COUNTIF(Model_Parameters!H:H,"No")</f>
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2358,7 +2301,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="36"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
         <v>20</v>
       </c>
@@ -2508,7 +2451,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
         <v>58</v>
       </c>
@@ -2558,7 +2501,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>67</v>
       </c>
@@ -2590,351 +2533,351 @@
         <v>74</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>76</v>
+        <v>47</v>
       </c>
       <c r="N5" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>61</v>
       </c>
       <c r="F6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="N6" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>87</v>
+        <v>47</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>61</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>47</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="L7" s="6" t="s">
         <v>45</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="F8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="G8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>101</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>103</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="N8" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O8" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G9" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="N9" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="O9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="P9" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="N9" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>70</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>87</v>
+        <v>47</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>47</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="P11" s="6" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>144</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>45</v>
@@ -2943,166 +2886,166 @@
         <v>46</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>148</v>
+        <v>46</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>149</v>
+        <v>47</v>
       </c>
       <c r="N12" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>150</v>
+        <v>47</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>70</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>84</v>
+        <v>143</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>158</v>
+        <v>47</v>
       </c>
       <c r="N13" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>159</v>
+        <v>47</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>166</v>
+        <v>47</v>
       </c>
       <c r="N14" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>167</v>
+        <v>47</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>61</v>
       </c>
       <c r="F15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="H15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="G15" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>84</v>
-      </c>
       <c r="I15" s="6" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>172</v>
+        <v>47</v>
       </c>
       <c r="N15" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>87</v>
+        <v>47</v>
       </c>
       <c r="P15" s="6" t="s">
         <v>47</v>
@@ -3110,31 +3053,31 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>45</v>
@@ -3143,16 +3086,16 @@
         <v>46</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>148</v>
+        <v>46</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>179</v>
+        <v>47</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>180</v>
+        <v>47</v>
       </c>
       <c r="P16" s="6" t="s">
         <v>47</v>
@@ -3160,216 +3103,216 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>70</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>84</v>
+        <v>169</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>186</v>
+        <v>47</v>
       </c>
       <c r="N17" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>159</v>
+        <v>47</v>
       </c>
       <c r="P17" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>193</v>
+        <v>46</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>194</v>
+        <v>47</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>196</v>
+        <v>47</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>197</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>198</v>
+        <v>179</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>199</v>
+        <v>180</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>200</v>
+        <v>181</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>201</v>
+        <v>182</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>75</v>
+        <v>184</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>45</v>
+        <v>185</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>205</v>
+        <v>47</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>47</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>206</v>
+        <v>189</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>208</v>
+        <v>191</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>209</v>
+        <v>192</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>70</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>210</v>
+        <v>193</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>212</v>
+        <v>47</v>
       </c>
       <c r="N20" s="6" t="s">
         <v>65</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>213</v>
+        <v>47</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>214</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>215</v>
+        <v>196</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>61</v>
@@ -3378,31 +3321,31 @@
         <v>70</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>218</v>
+        <v>199</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>45</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>193</v>
+        <v>46</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>219</v>
+        <v>47</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>221</v>
+        <v>47</v>
       </c>
       <c r="P21" s="6" t="s">
         <v>47</v>
@@ -3410,52 +3353,52 @@
     </row>
     <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>41</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>47</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>228</v>
+        <v>207</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>47</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>229</v>
+        <v>208</v>
       </c>
       <c r="L22" s="6" t="s">
         <v>45</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>230</v>
+        <v>209</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>232</v>
+        <v>211</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>233</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -3503,51 +3446,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>234</v>
+        <v>213</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>235</v>
+        <v>214</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>236</v>
+        <v>215</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>237</v>
+        <v>216</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>238</v>
+        <v>217</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>239</v>
+        <v>218</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>240</v>
+        <v>219</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>241</v>
+        <v>220</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>242</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>243</v>
+        <v>222</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>244</v>
+        <v>223</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>245</v>
+        <v>224</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>246</v>
+        <v>225</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>247</v>
+        <v>226</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>248</v>
+        <v>227</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>47</v>
@@ -3556,143 +3499,143 @@
         <v>46</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>250</v>
+        <v>229</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>251</v>
+        <v>230</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>252</v>
+        <v>231</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>253</v>
+        <v>232</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>254</v>
+        <v>233</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>255</v>
+        <v>234</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>257</v>
+        <v>236</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>258</v>
+        <v>237</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>259</v>
+        <v>238</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>260</v>
+        <v>239</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>261</v>
+        <v>240</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>262</v>
+        <v>241</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>263</v>
+        <v>242</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>46</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>264</v>
+        <v>243</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>258</v>
+        <v>237</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>265</v>
+        <v>244</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>266</v>
+        <v>245</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>267</v>
+        <v>246</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>263</v>
+        <v>242</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>46</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>270</v>
+        <v>249</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>271</v>
+        <v>250</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>272</v>
+        <v>251</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>274</v>
+        <v>253</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>148</v>
+        <v>46</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>278</v>
-      </c>
       <c r="F7" s="6" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>58</v>
@@ -3701,752 +3644,752 @@
         <v>46</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="G11" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="B12" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="E12" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>287</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="H12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="B13" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="H13" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="B14" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>301</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>303</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>304</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>308</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>310</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>311</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>312</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>315</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>316</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>318</v>
-      </c>
       <c r="G14" s="6" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>256</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="G18" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="B19" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G19" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="H15" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="I15" s="6" t="s">
+      <c r="B20" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="F20" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="H20" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="B21" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="H16" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="G21" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="B22" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="G22" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D18" s="6" t="s">
+      <c r="B23" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="G18" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="G23" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="B24" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="G19" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D20" s="6" t="s">
+      <c r="G24" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="H24" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>336</v>
-      </c>
-      <c r="G20" s="6" t="s">
+      <c r="B25" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="H20" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G25" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="B26" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D22" s="6" t="s">
+      <c r="D26" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="G26" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="H26" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>328</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="B27" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="D27" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="G27" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C24" s="6" t="s">
+      <c r="H27" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="B28" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="D28" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F28" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G28" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="H24" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+      <c r="H28" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C25" s="6" t="s">
+      <c r="B29" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="G25" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
+      <c r="G29" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C26" s="6" t="s">
+      <c r="B30" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="E26" s="6" t="s">
+      <c r="D30" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="H26" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="G30" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C27" s="6" t="s">
+      <c r="B31" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="E27" s="6" t="s">
+      <c r="E31" s="6" t="s">
         <v>379</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F31" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="G31" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="H27" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="B32" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C32" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C28" s="6" t="s">
+      <c r="D32" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="E28" s="6" t="s">
+      <c r="E32" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F32" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G32" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="H28" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>390</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>391</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>392</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>393</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>394</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>395</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I30" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>397</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>399</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>400</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
-        <v>401</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>402</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>403</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>404</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>405</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>406</v>
-      </c>
       <c r="H32" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>144</v>
+        <v>254</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>407</v>
+        <v>387</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>244</v>
+        <v>223</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>408</v>
+        <v>388</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>409</v>
+        <v>389</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>411</v>
+        <v>391</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>47</v>
@@ -4455,7 +4398,7 @@
         <v>46</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -4488,41 +4431,42 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>412</v>
+        <v>392</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>413</v>
+        <v>393</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>414</v>
+        <v>394</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>415</v>
+        <v>395</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>416</v>
+        <v>396</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>417</v>
+        <v>397</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>418</v>
+        <v>398</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>419</v>
+        <v>399</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>47</v>
@@ -4531,103 +4475,103 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>420</v>
+        <v>400</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>421</v>
+        <v>401</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>422</v>
+        <v>402</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>423</v>
+        <v>47</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>424</v>
+        <v>403</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>425</v>
+        <v>404</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>426</v>
+        <v>399</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>426</v>
+        <v>47</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>428</v>
+        <v>405</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>423</v>
+        <v>47</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>430</v>
+        <v>408</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>431</v>
+        <v>409</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>423</v>
+        <v>47</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>432</v>
+        <v>411</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>433</v>
+        <v>412</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>45</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>434</v>
+        <v>415</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>435</v>
+        <v>416</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>47</v>
+        <v>418</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>45</v>
@@ -4635,13 +4579,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>47</v>
@@ -4652,74 +4596,40 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>437</v>
+        <v>421</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>438</v>
+        <v>422</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>47</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>45</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>439</v>
+        <v>424</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>440</v>
+        <v>425</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>47</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>441</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>442</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>422</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>443</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>445</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E13">
+  <conditionalFormatting sqref="E2:E11">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Yes"</formula>
     </cfRule>
@@ -4762,25 +4672,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>446</v>
+        <v>427</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>447</v>
+        <v>428</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>448</v>
+        <v>429</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>449</v>
+        <v>430</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>450</v>
+        <v>431</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>451</v>
+        <v>432</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>452</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4788,22 +4698,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>453</v>
+        <v>434</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>454</v>
+        <v>435</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>455</v>
+        <v>436</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>456</v>
+        <v>437</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>457</v>
+        <v>438</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4811,22 +4721,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>453</v>
+        <v>434</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>458</v>
+        <v>439</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>459</v>
+        <v>440</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>58</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>460</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4834,22 +4744,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>453</v>
+        <v>434</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>461</v>
+        <v>442</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>462</v>
+        <v>443</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>463</v>
+        <v>444</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>464</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4857,45 +4767,45 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>453</v>
+        <v>434</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>465</v>
+        <v>446</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>466</v>
+        <v>447</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>47</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>468</v>
+        <v>449</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>469</v>
+        <v>450</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>470</v>
+        <v>451</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>471</v>
+        <v>452</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>221</v>
+        <v>117</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>472</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4903,22 +4813,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>473</v>
+        <v>454</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>474</v>
+        <v>455</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>475</v>
+        <v>456</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>221</v>
+        <v>117</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>476</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4926,22 +4836,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>473</v>
+        <v>454</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>431</v>
+        <v>416</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>477</v>
+        <v>458</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>478</v>
+        <v>459</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>479</v>
+        <v>117</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>480</v>
+        <v>460</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4949,22 +4859,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>473</v>
+        <v>454</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>481</v>
+        <v>461</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>483</v>
+        <v>463</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>221</v>
+        <v>117</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>484</v>
+        <v>464</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4972,22 +4882,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>473</v>
+        <v>454</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>485</v>
+        <v>465</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>486</v>
+        <v>466</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>67</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>487</v>
+        <v>467</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>488</v>
+        <v>468</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4995,22 +4905,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>489</v>
+        <v>469</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>490</v>
+        <v>470</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>491</v>
+        <v>471</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>492</v>
+        <v>472</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>493</v>
+        <v>473</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5018,22 +4928,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>494</v>
+        <v>474</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>495</v>
+        <v>475</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>496</v>
+        <v>476</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>492</v>
+        <v>472</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>497</v>
+        <v>477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5041,22 +4951,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>498</v>
+        <v>478</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>499</v>
+        <v>479</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>492</v>
+        <v>472</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>501</v>
+        <v>481</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>502</v>
+        <v>482</v>
       </c>
     </row>
   </sheetData>
@@ -5090,53 +5000,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>503</v>
+        <v>483</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>504</v>
+        <v>484</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>505</v>
+        <v>485</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>506</v>
+        <v>486</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>508</v>
+        <v>488</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>509</v>
+        <v>489</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>510</v>
+        <v>490</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>512</v>
+        <v>492</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>513</v>
+        <v>493</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>514</v>
+        <v>494</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>515</v>
+        <v>495</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5144,16 +5054,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>516</v>
+        <v>496</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>517</v>
+        <v>497</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>518</v>
+        <v>498</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>519</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5161,16 +5071,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>520</v>
+        <v>500</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>521</v>
+        <v>501</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>522</v>
+        <v>503</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5178,16 +5088,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>523</v>
+        <v>504</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>524</v>
+        <v>505</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>514</v>
+        <v>494</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>522</v>
+        <v>503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FotMob 2017-18 to 2019-20 and refresh workbook counts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019genJUXM7TYZhfbpNvVXCS
</commit_message>
<xml_diff>
--- a/FantaBall-Complete/docs/Data-Sources-and-Calibration-Plan.xlsx
+++ b/FantaBall-Complete/docs/Data-Sources-and-Calibration-Plan.xlsx
@@ -778,7 +778,7 @@
     <t xml:space="preserve">FotMob</t>
   </si>
   <si>
-    <t xml:space="preserve">2018-19 → 2026-27</t>
+    <t xml:space="preserve">2017-18 → 2026-27</t>
   </si>
   <si>
     <t xml:space="preserve">Formations, minutes, age</t>
@@ -3876,10 +3876,10 @@
         <v>250</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>141869</v>
+        <v>158770</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>251</v>
@@ -3896,10 +3896,10 @@
         <v>250</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>7630</v>
+        <v>7878</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>253</v>

</xml_diff>